<commit_message>
Update team decision tree analysis docs
</commit_message>
<xml_diff>
--- a/team/jin-qinhao/Take-Home-Exercise2/data/tourism_four_part_analysis_ready.xlsx
+++ b/team/jin-qinhao/Take-Home-Exercise2/data/tourism_four_part_analysis_ready.xlsx
@@ -607,6 +607,9 @@
       <c r="C5">
         <v>84.67200801</v>
       </c>
+      <c r="E5">
+        <v>6724.5678785</v>
+      </c>
       <c r="G5">
         <v>1480161</v>
       </c>
@@ -745,6 +748,9 @@
       <c r="C8">
         <v>83.7548828</v>
       </c>
+      <c r="E8">
+        <v>13404.76334795</v>
+      </c>
       <c r="G8">
         <v>1387601</v>
       </c>
@@ -883,6 +889,9 @@
       <c r="C11">
         <v>84.33686469</v>
       </c>
+      <c r="E11">
+        <v>20345.77697974</v>
+      </c>
       <c r="G11">
         <v>1320050</v>
       </c>
@@ -1168,6 +1177,9 @@
       <c r="C17">
         <v>87.20196257000001</v>
       </c>
+      <c r="E17">
+        <v>6867.78782354</v>
+      </c>
       <c r="G17">
         <v>1584406</v>
       </c>
@@ -1306,6 +1318,9 @@
       <c r="C20">
         <v>85.46062713000001</v>
       </c>
+      <c r="E20">
+        <v>13461.72489445</v>
+      </c>
       <c r="G20">
         <v>1544679</v>
       </c>
@@ -1444,6 +1459,9 @@
       <c r="C23">
         <v>85.33643060999999</v>
       </c>
+      <c r="E23">
+        <v>20610.56743432</v>
+      </c>
       <c r="G23">
         <v>1415149</v>
       </c>
@@ -1729,6 +1747,9 @@
       <c r="C29">
         <v>84.31584076999999</v>
       </c>
+      <c r="E29">
+        <v>6600.12739729</v>
+      </c>
       <c r="G29">
         <v>1564664</v>
       </c>
@@ -1867,6 +1888,9 @@
       <c r="C32">
         <v>86.14354211</v>
       </c>
+      <c r="E32">
+        <v>13165.79436414</v>
+      </c>
       <c r="G32">
         <v>1551847</v>
       </c>
@@ -2005,6 +2029,9 @@
       <c r="C35">
         <v>87.13118264000001</v>
       </c>
+      <c r="E35">
+        <v>20548.88298768</v>
+      </c>
       <c r="G35">
         <v>1463543</v>
       </c>
@@ -2290,6 +2317,9 @@
       <c r="C41">
         <v>40.16224463</v>
       </c>
+      <c r="E41">
+        <v>4029.34738486</v>
+      </c>
       <c r="G41">
         <v>240001</v>
       </c>
@@ -2428,6 +2458,9 @@
       <c r="C44">
         <v>57.04914877</v>
       </c>
+      <c r="E44">
+        <v>4186.55740391</v>
+      </c>
       <c r="G44">
         <v>2171</v>
       </c>
@@ -2566,6 +2599,9 @@
       <c r="C47">
         <v>63.12299737</v>
       </c>
+      <c r="E47">
+        <v>4435.65426399</v>
+      </c>
       <c r="G47">
         <v>9500</v>
       </c>
@@ -2851,6 +2887,9 @@
       <c r="C53">
         <v>51.42837194</v>
       </c>
+      <c r="E53">
+        <v>424.51831782</v>
+      </c>
       <c r="G53">
         <v>27202</v>
       </c>
@@ -2989,6 +3028,9 @@
       <c r="C56">
         <v>54.64458579</v>
       </c>
+      <c r="E56">
+        <v>827.64269004</v>
+      </c>
       <c r="G56">
         <v>10029</v>
       </c>
@@ -3127,6 +3169,9 @@
       <c r="C59">
         <v>65.10329204999999</v>
       </c>
+      <c r="E59">
+        <v>1189.70586264</v>
+      </c>
       <c r="G59">
         <v>19009</v>
       </c>
@@ -3412,6 +3457,9 @@
       <c r="C65">
         <v>60.58287962</v>
       </c>
+      <c r="E65">
+        <v>1417.14408657</v>
+      </c>
       <c r="G65">
         <v>121207</v>
       </c>
@@ -3550,6 +3598,9 @@
       <c r="C68">
         <v>78.07311692</v>
       </c>
+      <c r="E68">
+        <v>4572.52438757</v>
+      </c>
       <c r="G68">
         <v>543733</v>
       </c>
@@ -3688,6 +3739,9 @@
       <c r="C71">
         <v>82.84273883</v>
       </c>
+      <c r="E71">
+        <v>9083.61939613</v>
+      </c>
       <c r="G71">
         <v>782215</v>
       </c>
@@ -3973,6 +4027,9 @@
       <c r="C77">
         <v>80.04863102</v>
       </c>
+      <c r="E77">
+        <v>6017.94372289</v>
+      </c>
       <c r="G77">
         <v>1021040</v>
       </c>
@@ -4111,6 +4168,9 @@
       <c r="C80">
         <v>81.06717027000001</v>
       </c>
+      <c r="E80">
+        <v>12445.99017278</v>
+      </c>
       <c r="G80">
         <v>1129310</v>
       </c>
@@ -4249,6 +4309,9 @@
       <c r="C83">
         <v>82.67366269</v>
       </c>
+      <c r="E83">
+        <v>20307.57071465</v>
+      </c>
       <c r="G83">
         <v>1130762</v>
       </c>
@@ -4534,6 +4597,9 @@
       <c r="C89">
         <v>83.41271879</v>
       </c>
+      <c r="E89">
+        <v>8077.16805887</v>
+      </c>
       <c r="G89">
         <v>1464865</v>
       </c>
@@ -4672,6 +4738,9 @@
       <c r="C92">
         <v>76.91959518</v>
       </c>
+      <c r="E92">
+        <v>14923.35371873</v>
+      </c>
       <c r="G92">
         <v>1250293</v>
       </c>
@@ -4810,6 +4879,9 @@
       <c r="C95">
         <v>83.09800989</v>
       </c>
+      <c r="E95">
+        <v>22421.03985439</v>
+      </c>
       <c r="G95">
         <v>1270681</v>
       </c>
@@ -4998,7 +5070,7 @@
         <v>45658</v>
       </c>
       <c r="B99">
-        <v>3.52215423</v>
+        <v>3.52215261</v>
       </c>
       <c r="C99">
         <v>81.80868991</v>
@@ -5030,7 +5102,7 @@
         <v>23.04757590320142</v>
       </c>
       <c r="O99">
-        <v>3.52215423</v>
+        <v>3.52215261</v>
       </c>
       <c r="P99">
         <v>1.633495</v>
@@ -5044,7 +5116,7 @@
         <v>45689</v>
       </c>
       <c r="B100">
-        <v>3.46523629</v>
+        <v>3.46523707</v>
       </c>
       <c r="C100">
         <v>83.82109185</v>
@@ -5076,7 +5148,7 @@
         <v>19.45346432302272</v>
       </c>
       <c r="O100">
-        <v>3.46523629</v>
+        <v>3.46523707</v>
       </c>
       <c r="P100">
         <v>1.377513</v>
@@ -5095,6 +5167,9 @@
       <c r="C101">
         <v>76.14225854999999</v>
       </c>
+      <c r="E101">
+        <v>8008.93668644</v>
+      </c>
       <c r="G101">
         <v>1296605</v>
       </c>
@@ -5182,7 +5257,7 @@
         <v>45778</v>
       </c>
       <c r="B103">
-        <v>3.56004101</v>
+        <v>3.56003864</v>
       </c>
       <c r="C103">
         <v>79.57640013</v>
@@ -5214,7 +5289,7 @@
         <v>17.61157644250711</v>
       </c>
       <c r="O103">
-        <v>3.56004101</v>
+        <v>3.56003864</v>
       </c>
       <c r="P103">
         <v>1.37417</v>
@@ -5233,6 +5308,9 @@
       <c r="C104">
         <v>75.02096415</v>
       </c>
+      <c r="E104">
+        <v>15594.03060042</v>
+      </c>
       <c r="G104">
         <v>1245947</v>
       </c>
@@ -5371,6 +5449,9 @@
       <c r="C107">
         <v>80.96374383</v>
       </c>
+      <c r="E107">
+        <v>23881.41968916</v>
+      </c>
       <c r="G107">
         <v>1254346</v>
       </c>
@@ -5464,10 +5545,10 @@
         <v>84.95384722999999</v>
       </c>
       <c r="G109">
-        <v>1293401</v>
+        <v>1293402</v>
       </c>
       <c r="H109">
-        <v>203531</v>
+        <v>203532</v>
       </c>
       <c r="I109">
         <v>2025</v>
@@ -5484,19 +5565,19 @@
         </is>
       </c>
       <c r="M109">
-        <v>0.1573610968292123</v>
+        <v>0.157361748319548</v>
       </c>
       <c r="N109">
-        <v>15.73610968292123</v>
+        <v>15.7361748319548</v>
       </c>
       <c r="O109">
         <v>3.29827077</v>
       </c>
       <c r="P109">
-        <v>1.293401</v>
+        <v>1.293402</v>
       </c>
       <c r="Q109">
-        <v>203.531</v>
+        <v>203.532</v>
       </c>
     </row>
     <row r="110">
@@ -5510,7 +5591,7 @@
         <v>76.44595653</v>
       </c>
       <c r="F110">
-        <v>3.48480057</v>
+        <v>3.48480029</v>
       </c>
       <c r="G110">
         <v>1363999</v>
@@ -5553,13 +5634,13 @@
         <v>46023</v>
       </c>
       <c r="B111">
-        <v>3.43209009</v>
+        <v>3.43208671</v>
       </c>
       <c r="C111">
         <v>81.17069512</v>
       </c>
       <c r="G111">
-        <v>1501420</v>
+        <v>1501426</v>
       </c>
       <c r="H111">
         <v>271953</v>
@@ -5579,16 +5660,16 @@
         </is>
       </c>
       <c r="M111">
-        <v>0.1811305297651556</v>
+        <v>0.1811298059311614</v>
       </c>
       <c r="N111">
-        <v>18.11305297651557</v>
+        <v>18.11298059311614</v>
       </c>
       <c r="O111">
-        <v>3.43209009</v>
+        <v>3.43208671</v>
       </c>
       <c r="P111">
-        <v>1.50142</v>
+        <v>1.501426</v>
       </c>
       <c r="Q111">
         <v>271.953</v>
@@ -11053,10 +11134,10 @@
         <v>81.80868991</v>
       </c>
       <c r="K99">
-        <v>3.52215423</v>
+        <v>3.52215261</v>
       </c>
       <c r="L99">
-        <v>3.52215423</v>
+        <v>3.52215261</v>
       </c>
       <c r="M99" t="inlineStr">
         <is>
@@ -11108,10 +11189,10 @@
         <v>83.82109185</v>
       </c>
       <c r="K100">
-        <v>3.46523629</v>
+        <v>3.46523707</v>
       </c>
       <c r="L100">
-        <v>3.46523629</v>
+        <v>3.46523707</v>
       </c>
       <c r="M100" t="inlineStr">
         <is>
@@ -11273,10 +11354,10 @@
         <v>79.57640013</v>
       </c>
       <c r="K103">
-        <v>3.56004101</v>
+        <v>3.56003864</v>
       </c>
       <c r="L103">
-        <v>3.56004101</v>
+        <v>3.56003864</v>
       </c>
       <c r="M103" t="inlineStr">
         <is>
@@ -11588,16 +11669,16 @@
         </is>
       </c>
       <c r="F109">
-        <v>1293401</v>
+        <v>1293402</v>
       </c>
       <c r="G109">
-        <v>203531</v>
+        <v>203532</v>
       </c>
       <c r="H109">
-        <v>0.1573610968292123</v>
+        <v>0.157361748319548</v>
       </c>
       <c r="I109">
-        <v>15.73610968292123</v>
+        <v>15.7361748319548</v>
       </c>
       <c r="J109">
         <v>84.95384722999999</v>
@@ -11698,25 +11779,25 @@
         </is>
       </c>
       <c r="F111">
-        <v>1501420</v>
+        <v>1501426</v>
       </c>
       <c r="G111">
         <v>271953</v>
       </c>
       <c r="H111">
-        <v>0.1811305297651556</v>
+        <v>0.1811298059311614</v>
       </c>
       <c r="I111">
-        <v>18.11305297651557</v>
+        <v>18.11298059311614</v>
       </c>
       <c r="J111">
         <v>81.17069512</v>
       </c>
       <c r="K111">
-        <v>3.43209009</v>
+        <v>3.43208671</v>
       </c>
       <c r="L111">
-        <v>3.43209009</v>
+        <v>3.43208671</v>
       </c>
       <c r="M111" t="inlineStr">
         <is>
@@ -11924,16 +12005,16 @@
         <v>226.02</v>
       </c>
       <c r="R2">
-        <v>0.76297296065819</v>
+        <v>0.7629727995952658</v>
       </c>
       <c r="S2">
-        <v>-0.2030058375629522</v>
+        <v>-0.2030058341489089</v>
       </c>
       <c r="T2">
         <v>0.2149550771338822</v>
       </c>
       <c r="U2">
-        <v>-0.5446409376964171</v>
+        <v>-0.544640929858071</v>
       </c>
       <c r="V2" t="inlineStr">
         <is>
@@ -11997,16 +12078,16 @@
         <v>316.805</v>
       </c>
       <c r="R3">
-        <v>0.7209186051686073</v>
+        <v>0.7209184472336083</v>
       </c>
       <c r="S3">
-        <v>0.3291853545365265</v>
+        <v>0.3291853633548724</v>
       </c>
       <c r="T3">
         <v>0.3854595728201931</v>
       </c>
       <c r="U3">
-        <v>-0.5137544200425357</v>
+        <v>-0.5137544123023888</v>
       </c>
       <c r="V3" t="inlineStr">
         <is>
@@ -12070,16 +12151,16 @@
         <v>268.993</v>
       </c>
       <c r="R4">
-        <v>0.5250818561534073</v>
+        <v>0.525081712784384</v>
       </c>
       <c r="S4">
-        <v>0.1930943502225197</v>
+        <v>0.1930943576588868</v>
       </c>
       <c r="T4">
         <v>0.8807125244281927</v>
       </c>
       <c r="U4">
-        <v>-0.5233195068540272</v>
+        <v>-0.5233194990834695</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
@@ -12107,6 +12188,9 @@
       <c r="C5">
         <v>84.67200801</v>
       </c>
+      <c r="E5">
+        <v>6724.5678785</v>
+      </c>
       <c r="G5">
         <v>1480161</v>
       </c>
@@ -12143,16 +12227,16 @@
         <v>264.711</v>
       </c>
       <c r="R5">
-        <v>0.7203973311461678</v>
+        <v>0.7203971732499402</v>
       </c>
       <c r="S5">
-        <v>0.03654821277651873</v>
+        <v>0.03654821862318888</v>
       </c>
       <c r="T5">
         <v>0.615242891830268</v>
       </c>
       <c r="U5">
-        <v>-0.5511437351663581</v>
+        <v>-0.5511437273073372</v>
       </c>
       <c r="V5" t="inlineStr">
         <is>
@@ -12216,16 +12300,16 @@
         <v>252.135</v>
       </c>
       <c r="R6">
-        <v>0.7049705706896305</v>
+        <v>0.7049704139408169</v>
       </c>
       <c r="S6">
-        <v>-0.02511480091715561</v>
+        <v>-0.0251147956966619</v>
       </c>
       <c r="T6">
         <v>0.6465903235551737</v>
       </c>
       <c r="U6">
-        <v>-0.5378703744340294</v>
+        <v>-0.5378703666172092</v>
       </c>
       <c r="V6" t="inlineStr">
         <is>
@@ -12289,16 +12373,16 @@
         <v>232.361</v>
       </c>
       <c r="R7">
-        <v>0.529814303017505</v>
+        <v>0.529814159296491</v>
       </c>
       <c r="S7">
-        <v>-0.03400192256535129</v>
+        <v>-0.03400191743510465</v>
       </c>
       <c r="T7">
         <v>0.4259200008385803</v>
       </c>
       <c r="U7">
-        <v>-0.5105200905651889</v>
+        <v>-0.5105200828353251</v>
       </c>
       <c r="V7" t="inlineStr">
         <is>
@@ -12326,6 +12410,9 @@
       <c r="C8">
         <v>83.7548828</v>
       </c>
+      <c r="E8">
+        <v>13404.76334795</v>
+      </c>
       <c r="G8">
         <v>1387601</v>
       </c>
@@ -12362,16 +12449,16 @@
         <v>218.118</v>
       </c>
       <c r="R8">
-        <v>0.5686705276335668</v>
+        <v>0.5686703810224987</v>
       </c>
       <c r="S8">
-        <v>-0.1436906212035279</v>
+        <v>-0.1436906171871496</v>
       </c>
       <c r="T8">
         <v>0.5426898743007261</v>
       </c>
       <c r="U8">
-        <v>-0.5025367389906025</v>
+        <v>-0.5025367312861206</v>
       </c>
       <c r="V8" t="inlineStr">
         <is>
@@ -12435,16 +12522,16 @@
         <v>349.654</v>
       </c>
       <c r="R9">
-        <v>0.9695171370777149</v>
+        <v>0.9695169606524164</v>
       </c>
       <c r="S9">
-        <v>0.3312074706358082</v>
+        <v>0.3312074794746883</v>
       </c>
       <c r="T9">
         <v>1.158335216813513</v>
       </c>
       <c r="U9">
-        <v>-0.5153281861261696</v>
+        <v>-0.5153281783810192</v>
       </c>
       <c r="V9" t="inlineStr">
         <is>
@@ -12508,16 +12595,16 @@
         <v>357.287</v>
       </c>
       <c r="R10">
-        <v>0.8500962091444824</v>
+        <v>0.8500960416014919</v>
       </c>
       <c r="S10">
-        <v>0.4552962612546418</v>
+        <v>0.4552962713536204</v>
       </c>
       <c r="T10">
         <v>0.9858169393613322</v>
       </c>
       <c r="U10">
-        <v>-0.5122932016846796</v>
+        <v>-0.5122931939491785</v>
       </c>
       <c r="V10" t="inlineStr">
         <is>
@@ -12545,6 +12632,9 @@
       <c r="C11">
         <v>84.33686469</v>
       </c>
+      <c r="E11">
+        <v>20345.77697974</v>
+      </c>
       <c r="G11">
         <v>1320050</v>
       </c>
@@ -12581,16 +12671,16 @@
         <v>226.978</v>
       </c>
       <c r="R11">
-        <v>0.457939139300813</v>
+        <v>0.4579390009257409</v>
       </c>
       <c r="S11">
-        <v>-0.02083895471189905</v>
+        <v>-0.02083894944798492</v>
       </c>
       <c r="T11">
         <v>0.5887299807187427</v>
       </c>
       <c r="U11">
-        <v>-0.5326461123197754</v>
+        <v>-0.5326461045195652</v>
       </c>
       <c r="V11" t="inlineStr">
         <is>
@@ -12654,16 +12744,16 @@
         <v>245.755</v>
       </c>
       <c r="R12">
-        <v>0.5927638785197834</v>
+        <v>0.5927637301166964</v>
       </c>
       <c r="S12">
-        <v>0.006677170454538808</v>
+        <v>0.006677175997874073</v>
       </c>
       <c r="T12">
         <v>0.4932110748447768</v>
       </c>
       <c r="U12">
-        <v>-0.5412855439576593</v>
+        <v>-0.5412855361299811</v>
       </c>
       <c r="V12" t="inlineStr">
         <is>
@@ -12727,16 +12817,16 @@
         <v>251.096</v>
       </c>
       <c r="R13">
-        <v>0.5846185621125437</v>
+        <v>0.5846184143152902</v>
       </c>
       <c r="S13">
-        <v>0.04368883155823413</v>
+        <v>0.04368883747741593</v>
       </c>
       <c r="T13">
         <v>0.6548109865645889</v>
       </c>
       <c r="U13">
-        <v>-0.5567549568565663</v>
+        <v>-0.5567549489797053</v>
       </c>
       <c r="V13" t="inlineStr">
         <is>
@@ -12809,16 +12899,16 @@
         <v>244.241</v>
       </c>
       <c r="R14">
-        <v>0.8670343364207973</v>
+        <v>0.8670341676179801</v>
       </c>
       <c r="S14">
-        <v>-0.15688798988209</v>
+        <v>-0.1568879859997285</v>
       </c>
       <c r="T14">
         <v>0.2173697525483227</v>
       </c>
       <c r="U14">
-        <v>-0.5436206393988744</v>
+        <v>-0.5436206315637722</v>
       </c>
       <c r="V14" t="inlineStr">
         <is>
@@ -12882,16 +12972,16 @@
         <v>291.208</v>
       </c>
       <c r="R15">
-        <v>0.8567776963000286</v>
+        <v>0.8567775282600815</v>
       </c>
       <c r="S15">
-        <v>0.09841936997212757</v>
+        <v>0.0984193764470878</v>
       </c>
       <c r="T15">
         <v>0.5162456948214821</v>
       </c>
       <c r="U15">
-        <v>-0.5284297085508359</v>
+        <v>-0.5284297007640311</v>
       </c>
       <c r="V15" t="inlineStr">
         <is>
@@ -12955,16 +13045,16 @@
         <v>366.616</v>
       </c>
       <c r="R16">
-        <v>0.7397549567153153</v>
+        <v>0.7397547973793034</v>
       </c>
       <c r="S16">
-        <v>0.593424510407612</v>
+        <v>0.5934245219092574</v>
       </c>
       <c r="T16">
         <v>0.878072644973563</v>
       </c>
       <c r="U16">
-        <v>-0.5308419471897441</v>
+        <v>-0.5308419393952698</v>
       </c>
       <c r="V16" t="inlineStr">
         <is>
@@ -12992,6 +13082,9 @@
       <c r="C17">
         <v>87.20196257000001</v>
       </c>
+      <c r="E17">
+        <v>6867.78782354</v>
+      </c>
       <c r="G17">
         <v>1584406</v>
       </c>
@@ -13028,16 +13121,16 @@
         <v>274.879</v>
       </c>
       <c r="R17">
-        <v>0.8912784961436945</v>
+        <v>0.8912783255376415</v>
       </c>
       <c r="S17">
-        <v>-0.007986332470507713</v>
+        <v>-0.007986327076077594</v>
       </c>
       <c r="T17">
         <v>0.8153855065345633</v>
       </c>
       <c r="U17">
-        <v>-0.5456582931766801</v>
+        <v>-0.5456582853350994</v>
       </c>
       <c r="V17" t="inlineStr">
         <is>
@@ -13101,16 +13194,16 @@
         <v>291.119</v>
       </c>
       <c r="R18">
-        <v>0.8254504389325987</v>
+        <v>0.8254502732227151</v>
       </c>
       <c r="S18">
-        <v>0.117131937018109</v>
+        <v>0.1171319436830918</v>
       </c>
       <c r="T18">
         <v>0.6600207362284128</v>
       </c>
       <c r="U18">
-        <v>-0.5454436153186815</v>
+        <v>-0.5454436074777833</v>
       </c>
       <c r="V18" t="inlineStr">
         <is>
@@ -13174,16 +13267,16 @@
         <v>264.802</v>
       </c>
       <c r="R19">
-        <v>0.7052017016241084</v>
+        <v>0.7052015448581037</v>
       </c>
       <c r="S19">
-        <v>0.046447139302115</v>
+        <v>0.0464471452493069</v>
       </c>
       <c r="T19">
         <v>0.4484215048849083</v>
       </c>
       <c r="U19">
-        <v>-0.5172372835376083</v>
+        <v>-0.5172372757863882</v>
       </c>
       <c r="V19" t="inlineStr">
         <is>
@@ -13211,6 +13304,9 @@
       <c r="C20">
         <v>85.46062713000001</v>
       </c>
+      <c r="E20">
+        <v>13461.72489445</v>
+      </c>
       <c r="G20">
         <v>1544679</v>
       </c>
@@ -13247,16 +13343,16 @@
         <v>242.118</v>
       </c>
       <c r="R20">
-        <v>0.8261569455479177</v>
+        <v>0.8261567797854855</v>
       </c>
       <c r="S20">
-        <v>-0.1474161360503294</v>
+        <v>-0.147416132071783</v>
       </c>
       <c r="T20">
         <v>0.6776298987663141</v>
       </c>
       <c r="U20">
-        <v>-0.5095611520975659</v>
+        <v>-0.509561144370751</v>
       </c>
       <c r="V20" t="inlineStr">
         <is>
@@ -13320,16 +13416,16 @@
         <v>361.019</v>
       </c>
       <c r="R21">
-        <v>1.134687236999206</v>
+        <v>1.13468704828886</v>
       </c>
       <c r="S21">
-        <v>0.2821002899892174</v>
+        <v>0.2821002983294232</v>
       </c>
       <c r="T21">
         <v>1.225487587123302</v>
       </c>
       <c r="U21">
-        <v>-0.5251121178330829</v>
+        <v>-0.5251121100568258</v>
       </c>
       <c r="V21" t="inlineStr">
         <is>
@@ -13393,16 +13489,16 @@
         <v>380.108</v>
       </c>
       <c r="R22">
-        <v>1.053096377902012</v>
+        <v>1.053096195260244</v>
       </c>
       <c r="S22">
-        <v>0.4278186272570462</v>
+        <v>0.4278186370769946</v>
       </c>
       <c r="T22">
         <v>1.15750592721214</v>
       </c>
       <c r="U22">
-        <v>-0.5165756175239495</v>
+        <v>-0.5165756097748331</v>
       </c>
       <c r="V22" t="inlineStr">
         <is>
@@ -13430,6 +13526,9 @@
       <c r="C23">
         <v>85.33643060999999</v>
       </c>
+      <c r="E23">
+        <v>20610.56743432</v>
+      </c>
       <c r="G23">
         <v>1415149</v>
       </c>
@@ -13466,16 +13565,16 @@
         <v>239.824</v>
       </c>
       <c r="R23">
-        <v>0.6138279388605021</v>
+        <v>0.6138277888907091</v>
       </c>
       <c r="S23">
-        <v>-0.04146523464514829</v>
+        <v>-0.0414652295906902</v>
       </c>
       <c r="T23">
         <v>0.6678048146944576</v>
       </c>
       <c r="U23">
-        <v>-0.5393800478532691</v>
+        <v>-0.5393800400316492</v>
       </c>
       <c r="V23" t="inlineStr">
         <is>
@@ -13539,16 +13638,16 @@
         <v>247.664</v>
       </c>
       <c r="R24">
-        <v>0.6994463774329596</v>
+        <v>0.6994462210950252</v>
       </c>
       <c r="S24">
-        <v>-0.04720453088922722</v>
+        <v>-0.04720452589305062</v>
       </c>
       <c r="T24">
         <v>0.7493928244989533</v>
       </c>
       <c r="U24">
-        <v>-0.5460777185407756</v>
+        <v>-0.5460777106978614</v>
       </c>
       <c r="V24" t="inlineStr">
         <is>
@@ -13612,16 +13711,16 @@
         <v>220.053</v>
       </c>
       <c r="R25">
-        <v>0.6004452938315817</v>
+        <v>0.6004451448571652</v>
       </c>
       <c r="S25">
-        <v>-0.1502706500400592</v>
+        <v>-0.1502706460904999</v>
       </c>
       <c r="T25">
         <v>0.6371965545646292</v>
       </c>
       <c r="U25">
-        <v>-0.5520921428943488</v>
+        <v>-0.5520921350323127</v>
       </c>
       <c r="V25" t="inlineStr">
         <is>
@@ -13694,16 +13793,16 @@
         <v>238.194</v>
       </c>
       <c r="R26">
-        <v>0.9221139855654267</v>
+        <v>0.9221138126658871</v>
       </c>
       <c r="S26">
-        <v>-0.2154427197676173</v>
+        <v>-0.2154427164798682</v>
       </c>
       <c r="T26">
         <v>0.3046245011891796</v>
       </c>
       <c r="U26">
-        <v>-0.5435115003260177</v>
+        <v>-0.5435114924912624</v>
       </c>
       <c r="V26" t="inlineStr">
         <is>
@@ -13767,16 +13866,16 @@
         <v>320.581</v>
       </c>
       <c r="R27">
-        <v>0.9571540909228744</v>
+        <v>0.9571539154171165</v>
       </c>
       <c r="S27">
-        <v>0.1904954704039624</v>
+        <v>0.1904954778139383</v>
       </c>
       <c r="T27">
         <v>0.6184959100999171</v>
       </c>
       <c r="U27">
-        <v>-0.5236453899749158</v>
+        <v>-0.523645382203322</v>
       </c>
       <c r="V27" t="inlineStr">
         <is>
@@ -13840,16 +13939,16 @@
         <v>339.55</v>
       </c>
       <c r="R28">
-        <v>0.751362319460267</v>
+        <v>0.7513621592609209</v>
       </c>
       <c r="S28">
-        <v>0.4334375025281324</v>
+        <v>0.4334375124051394</v>
       </c>
       <c r="T28">
         <v>0.9165243194051609</v>
       </c>
       <c r="U28">
-        <v>-0.5195240900688828</v>
+        <v>-0.519524082310392</v>
       </c>
       <c r="V28" t="inlineStr">
         <is>
@@ -13877,6 +13976,9 @@
       <c r="C29">
         <v>84.31584076999999</v>
       </c>
+      <c r="E29">
+        <v>6600.12739729</v>
+      </c>
       <c r="G29">
         <v>1564664</v>
       </c>
@@ -13913,16 +14015,16 @@
         <v>300.209</v>
       </c>
       <c r="R29">
-        <v>0.8589168868638137</v>
+        <v>0.8589167186647575</v>
       </c>
       <c r="S29">
-        <v>0.1450206761888326</v>
+        <v>0.1450206831370205</v>
       </c>
       <c r="T29">
         <v>0.5870667957799054</v>
       </c>
       <c r="U29">
-        <v>-0.5523815573024486</v>
+        <v>-0.5523815494394922</v>
       </c>
       <c r="V29" t="inlineStr">
         <is>
@@ -13986,16 +14088,16 @@
         <v>302.098</v>
       </c>
       <c r="R30">
-        <v>0.9114704879940425</v>
+        <v>0.9114703158861466</v>
       </c>
       <c r="S30">
-        <v>0.1227962060658227</v>
+        <v>0.1227962127883251</v>
       </c>
       <c r="T30">
         <v>0.6748043714405194</v>
       </c>
       <c r="U30">
-        <v>-0.5434728675671308</v>
+        <v>-0.5434728597324983</v>
       </c>
       <c r="V30" t="inlineStr">
         <is>
@@ -14059,16 +14161,16 @@
         <v>283.445</v>
       </c>
       <c r="R31">
-        <v>0.7329046292317463</v>
+        <v>0.732904470405249</v>
       </c>
       <c r="S31">
-        <v>0.1337474052931108</v>
+        <v>0.1337474121268206</v>
       </c>
       <c r="T31">
         <v>0.4032039376824735</v>
       </c>
       <c r="U31">
-        <v>-0.5123656070179055</v>
+        <v>-0.5123655992821742</v>
       </c>
       <c r="V31" t="inlineStr">
         <is>
@@ -14096,6 +14198,9 @@
       <c r="C32">
         <v>86.14354211</v>
       </c>
+      <c r="E32">
+        <v>13165.79436414</v>
+      </c>
       <c r="G32">
         <v>1551847</v>
       </c>
@@ -14132,16 +14237,16 @@
         <v>266.107</v>
       </c>
       <c r="R32">
-        <v>0.8379069209971217</v>
+        <v>0.837906754360748</v>
       </c>
       <c r="S32">
-        <v>-0.02474299230206999</v>
+        <v>-0.02474298707780064</v>
       </c>
       <c r="T32">
         <v>0.7316547385317879</v>
       </c>
       <c r="U32">
-        <v>-0.5023678934475863</v>
+        <v>-0.5023678857436412</v>
       </c>
       <c r="V32" t="inlineStr">
         <is>
@@ -14205,16 +14310,16 @@
         <v>389.503</v>
       </c>
       <c r="R33">
-        <v>1.248936405370184</v>
+        <v>1.248936208162196</v>
       </c>
       <c r="S33">
-        <v>0.3465951791610201</v>
+        <v>0.3465951881561595</v>
       </c>
       <c r="T33">
         <v>1.345370760187991</v>
       </c>
       <c r="U33">
-        <v>-0.5216939127327783</v>
+        <v>-0.521693904967389</v>
       </c>
       <c r="V33" t="inlineStr">
         <is>
@@ -14278,16 +14383,16 @@
         <v>397.07</v>
       </c>
       <c r="R34">
-        <v>1.139942597112228</v>
+        <v>1.139942408010999</v>
       </c>
       <c r="S34">
-        <v>0.4517834838203089</v>
+        <v>0.451783493883616</v>
       </c>
       <c r="T34">
         <v>1.22989168500685</v>
       </c>
       <c r="U34">
-        <v>-0.5091222411445817</v>
+        <v>-0.5091222334191622</v>
       </c>
       <c r="V34" t="inlineStr">
         <is>
@@ -14315,6 +14420,9 @@
       <c r="C35">
         <v>87.13118264000001</v>
       </c>
+      <c r="E35">
+        <v>20548.88298768</v>
+      </c>
       <c r="G35">
         <v>1463543</v>
       </c>
@@ -14351,16 +14459,16 @@
         <v>248.568</v>
       </c>
       <c r="R35">
-        <v>0.6931566654074858</v>
+        <v>0.6931565095373686</v>
       </c>
       <c r="S35">
-        <v>-0.03837790248801308</v>
+        <v>-0.0383778974022037</v>
       </c>
       <c r="T35">
         <v>0.8097861647587224</v>
       </c>
       <c r="U35">
-        <v>-0.5360419206132656</v>
+        <v>-0.5360419128022588</v>
       </c>
       <c r="V35" t="inlineStr">
         <is>
@@ -14424,16 +14532,16 @@
         <v>258.611</v>
       </c>
       <c r="R36">
-        <v>0.8028799294515594</v>
+        <v>0.8028797654204285</v>
       </c>
       <c r="S36">
-        <v>-0.04558796734333045</v>
+        <v>-0.04558796233073795</v>
       </c>
       <c r="T36">
         <v>0.7933538848739009</v>
       </c>
       <c r="U36">
-        <v>-0.539198560529891</v>
+        <v>-0.5391985527088482</v>
       </c>
       <c r="V36" t="inlineStr">
         <is>
@@ -14497,16 +14605,16 @@
         <v>248.636</v>
       </c>
       <c r="R37">
-        <v>0.808107422714326</v>
+        <v>0.8081072582943839</v>
       </c>
       <c r="S37">
-        <v>-0.1026633866018611</v>
+        <v>-0.1026633821688589</v>
       </c>
       <c r="T37">
         <v>0.9437751197520571</v>
       </c>
       <c r="U37">
-        <v>-0.5536211602150504</v>
+        <v>-0.5536211523481529</v>
       </c>
       <c r="V37" t="inlineStr">
         <is>
@@ -14579,16 +14687,16 @@
         <v>272.742</v>
       </c>
       <c r="R38">
-        <v>1.121679974835501</v>
+        <v>1.121679787092612</v>
       </c>
       <c r="S38">
-        <v>-0.1359963903658607</v>
+        <v>-0.1359963862713489</v>
       </c>
       <c r="T38">
         <v>0.4818741796557495</v>
       </c>
       <c r="U38">
-        <v>-0.5533657670987874</v>
+        <v>-0.5533657592327019</v>
       </c>
       <c r="V38" t="inlineStr">
         <is>
@@ -14652,16 +14760,16 @@
         <v>329.047</v>
       </c>
       <c r="R39">
-        <v>1.061259725800594</v>
+        <v>1.061259542551652</v>
       </c>
       <c r="S39">
-        <v>0.1704409632674765</v>
+        <v>0.1704409704738026</v>
       </c>
       <c r="T39">
         <v>0.4790390880308563</v>
       </c>
       <c r="U39">
-        <v>-0.5163594524576338</v>
+        <v>-0.5163594447092046</v>
       </c>
       <c r="V39" t="inlineStr">
         <is>
@@ -14725,16 +14833,16 @@
         <v>6.222</v>
       </c>
       <c r="R40">
-        <v>-0.5044245028058396</v>
+        <v>-0.5044245696020819</v>
       </c>
       <c r="S40">
-        <v>-1.381731406375385</v>
+        <v>-1.381731414931081</v>
       </c>
       <c r="T40">
         <v>-2.202158098359493</v>
       </c>
       <c r="U40">
-        <v>-0.4596757765242265</v>
+        <v>-0.4596757689560151</v>
       </c>
       <c r="V40" t="inlineStr">
         <is>
@@ -14762,6 +14870,9 @@
       <c r="C41">
         <v>40.16224463</v>
       </c>
+      <c r="E41">
+        <v>4029.34738486</v>
+      </c>
       <c r="G41">
         <v>240001</v>
       </c>
@@ -14798,16 +14909,16 @@
         <v>1.488</v>
       </c>
       <c r="R41">
-        <v>-1.312505787308749</v>
+        <v>-1.312505794001398</v>
       </c>
       <c r="S41">
-        <v>-1.400787358585541</v>
+        <v>-1.400787367334746</v>
       </c>
       <c r="T41">
         <v>-2.905887710113297</v>
       </c>
       <c r="U41">
-        <v>-0.2790193245277154</v>
+        <v>-0.2790193175338756</v>
       </c>
       <c r="V41" t="inlineStr">
         <is>
@@ -14871,16 +14982,16 @@
         <v>0.018</v>
       </c>
       <c r="R42">
-        <v>-1.70469236322916</v>
+        <v>-1.704692340751696</v>
       </c>
       <c r="S42">
-        <v>-1.252590498540637</v>
+        <v>-1.25259050578493</v>
       </c>
       <c r="T42">
         <v>-2.884409141476965</v>
       </c>
       <c r="U42">
-        <v>2.576285806954851</v>
+        <v>2.576285804870653</v>
       </c>
       <c r="V42" t="inlineStr">
         <is>
@@ -14944,16 +15055,16 @@
         <v>0.023</v>
       </c>
       <c r="R43">
-        <v>-1.704479263786025</v>
+        <v>-1.704479241324411</v>
       </c>
       <c r="S43">
-        <v>-1.234803873634046</v>
+        <v>-1.23480388069772</v>
       </c>
       <c r="T43">
         <v>-1.395434164901923</v>
       </c>
       <c r="U43">
-        <v>2.576285806954851</v>
+        <v>2.576285804870653</v>
       </c>
       <c r="V43" t="inlineStr">
         <is>
@@ -14981,6 +15092,9 @@
       <c r="C44">
         <v>57.04914877</v>
       </c>
+      <c r="E44">
+        <v>4186.55740391</v>
+      </c>
       <c r="G44">
         <v>2171</v>
       </c>
@@ -15017,16 +15131,16 @@
         <v>0.118</v>
       </c>
       <c r="R44">
-        <v>-1.702363022393039</v>
+        <v>-1.702363000088827</v>
       </c>
       <c r="S44">
-        <v>-0.9998833083392099</v>
+        <v>-0.999883313017309</v>
       </c>
       <c r="T44">
         <v>-1.569978677486094</v>
       </c>
       <c r="U44">
-        <v>2.576285806954851</v>
+        <v>2.576285804870653</v>
       </c>
       <c r="V44" t="inlineStr">
         <is>
@@ -15090,16 +15204,16 @@
         <v>0.958</v>
       </c>
       <c r="R45">
-        <v>-1.69470455625204</v>
+        <v>-1.694704534517451</v>
       </c>
       <c r="S45">
-        <v>-0.2868389433412005</v>
+        <v>-0.2868389407784668</v>
       </c>
       <c r="T45">
         <v>-0.8309139960845137</v>
       </c>
       <c r="U45">
-        <v>2.576285806954851</v>
+        <v>2.576285804870653</v>
       </c>
       <c r="V45" t="inlineStr">
         <is>
@@ -15163,16 +15277,16 @@
         <v>2.163</v>
       </c>
       <c r="R46">
-        <v>-1.691312996653211</v>
+        <v>-1.69131297517088</v>
       </c>
       <c r="S46">
-        <v>0.5682838878677273</v>
+        <v>0.5682838991140743</v>
       </c>
       <c r="T46">
         <v>-0.9603786017126557</v>
       </c>
       <c r="U46">
-        <v>2.576285806954851</v>
+        <v>2.576285804870653</v>
       </c>
       <c r="V46" t="inlineStr">
         <is>
@@ -15200,6 +15314,9 @@
       <c r="C47">
         <v>63.12299737</v>
       </c>
+      <c r="E47">
+        <v>4435.65426399</v>
+      </c>
       <c r="G47">
         <v>9500</v>
       </c>
@@ -15236,16 +15353,16 @@
         <v>2.422</v>
       </c>
       <c r="R47">
-        <v>-1.690349131479644</v>
+        <v>-1.690349110069003</v>
       </c>
       <c r="S47">
-        <v>0.6701974320109992</v>
+        <v>0.6701974442922594</v>
       </c>
       <c r="T47">
         <v>-1.089481533647266</v>
       </c>
       <c r="U47">
-        <v>2.576285806954851</v>
+        <v>2.576285804870653</v>
       </c>
       <c r="V47" t="inlineStr">
         <is>
@@ -15309,16 +15426,16 @@
         <v>3.169</v>
       </c>
       <c r="R48">
-        <v>-1.683957787412059</v>
+        <v>-1.683957766476795</v>
       </c>
       <c r="S48">
-        <v>0.5166958375887851</v>
+        <v>0.5166958483112651</v>
       </c>
       <c r="T48">
         <v>-1.527127240353666</v>
       </c>
       <c r="U48">
-        <v>1.927163585844242</v>
+        <v>1.927163585823835</v>
       </c>
       <c r="V48" t="inlineStr">
         <is>
@@ -15382,16 +15499,16 @@
         <v>4.007</v>
       </c>
       <c r="R49">
-        <v>-1.681744831656419</v>
+        <v>-1.68174481088575</v>
       </c>
       <c r="S49">
-        <v>0.8095028400355017</v>
+        <v>0.8095028537313823</v>
       </c>
       <c r="T49">
         <v>-1.797880320721621</v>
       </c>
       <c r="U49">
-        <v>1.479587105252192</v>
+        <v>1.479587106654792</v>
       </c>
       <c r="V49" t="inlineStr">
         <is>
@@ -15464,16 +15581,16 @@
         <v>7.657</v>
       </c>
       <c r="R50">
-        <v>-1.666301678935026</v>
+        <v>-1.66630165931299</v>
       </c>
       <c r="S50">
-        <v>1.185141764724753</v>
+        <v>1.185141782235177</v>
       </c>
       <c r="T50">
         <v>-1.174529948793503</v>
       </c>
       <c r="U50">
-        <v>1.210340694482536</v>
+        <v>1.210340696741166</v>
       </c>
       <c r="V50" t="inlineStr">
         <is>
@@ -15537,16 +15654,16 @@
         <v>6.599</v>
       </c>
       <c r="R51">
-        <v>-1.667619617029495</v>
+        <v>-1.667619597309434</v>
       </c>
       <c r="S51">
-        <v>0.8989158984003619</v>
+        <v>0.8989159130042155</v>
       </c>
       <c r="T51">
         <v>-2.577503332490576</v>
       </c>
       <c r="U51">
-        <v>1.478249621810847</v>
+        <v>1.478249623217699</v>
       </c>
       <c r="V51" t="inlineStr">
         <is>
@@ -15610,16 +15727,16 @@
         <v>4.498</v>
       </c>
       <c r="R52">
-        <v>-1.676184575417064</v>
+        <v>-1.676184555059957</v>
       </c>
       <c r="S52">
-        <v>0.6119117896736453</v>
+        <v>0.6119118013630256</v>
       </c>
       <c r="T52">
         <v>-2.588863576752217</v>
       </c>
       <c r="U52">
-        <v>1.799482795790473</v>
+        <v>1.799482796176009</v>
       </c>
       <c r="V52" t="inlineStr">
         <is>
@@ -15647,6 +15764,9 @@
       <c r="C53">
         <v>51.42837194</v>
       </c>
+      <c r="E53">
+        <v>424.51831782</v>
+      </c>
       <c r="G53">
         <v>27202</v>
       </c>
@@ -15683,16 +15803,16 @@
         <v>8.891999999999999</v>
       </c>
       <c r="R53">
-        <v>-1.661331544230507</v>
+        <v>-1.661331524978141</v>
       </c>
       <c r="S53">
-        <v>1.269147996745575</v>
+        <v>1.269148015109067</v>
       </c>
       <c r="T53">
         <v>-2.014633687979847</v>
       </c>
       <c r="U53">
-        <v>1.925822958776817</v>
+        <v>1.925822958760673</v>
       </c>
       <c r="V53" t="inlineStr">
         <is>
@@ -15756,16 +15876,16 @@
         <v>9.055999999999999</v>
       </c>
       <c r="R54">
-        <v>-1.663733011031998</v>
+        <v>-1.663732991601015</v>
       </c>
       <c r="S54">
-        <v>1.477116454156138</v>
+        <v>1.477116474631511</v>
       </c>
       <c r="T54">
         <v>-1.913893329821995</v>
       </c>
       <c r="U54">
-        <v>2.071981674066807</v>
+        <v>2.071981673585972</v>
       </c>
       <c r="V54" t="inlineStr">
         <is>
@@ -15829,16 +15949,16 @@
         <v>7.388</v>
       </c>
       <c r="R55">
-        <v>-1.682661159261903</v>
+        <v>-1.682661138423079</v>
       </c>
       <c r="S55">
-        <v>2.882331877566948</v>
+        <v>2.882331912312023</v>
       </c>
       <c r="T55">
         <v>-1.895090550667504</v>
       </c>
       <c r="U55">
-        <v>2.00519746536107</v>
+        <v>2.005197465092567</v>
       </c>
       <c r="V55" t="inlineStr">
         <is>
@@ -15866,6 +15986,9 @@
       <c r="C56">
         <v>54.64458579</v>
       </c>
+      <c r="E56">
+        <v>827.64269004</v>
+      </c>
       <c r="G56">
         <v>10029</v>
       </c>
@@ -15902,16 +16025,16 @@
         <v>6.983</v>
       </c>
       <c r="R56">
-        <v>-1.68948198066873</v>
+        <v>-1.689481959322586</v>
       </c>
       <c r="S56">
-        <v>4.34458685647554</v>
+        <v>4.344586906069541</v>
       </c>
       <c r="T56">
         <v>-1.760201667909428</v>
       </c>
       <c r="U56">
-        <v>2.568080307587826</v>
+        <v>2.568080305529715</v>
       </c>
       <c r="V56" t="inlineStr">
         <is>
@@ -15975,16 +16098,16 @@
         <v>12.669</v>
       </c>
       <c r="R57">
-        <v>-1.675568226258456</v>
+        <v>-1.675568205947192</v>
       </c>
       <c r="S57">
-        <v>4.243857407158814</v>
+        <v>4.243857455729927</v>
       </c>
       <c r="T57">
         <v>-1.645978267327267</v>
       </c>
       <c r="U57">
-        <v>2.11789767840994</v>
+        <v>2.117897677783121</v>
       </c>
       <c r="V57" t="inlineStr">
         <is>
@@ -16048,16 +16171,16 @@
         <v>8.907</v>
       </c>
       <c r="R58">
-        <v>-1.679879391915739</v>
+        <v>-1.679879371283818</v>
       </c>
       <c r="S58">
-        <v>3.215347439374033</v>
+        <v>3.215347477500818</v>
       </c>
       <c r="T58">
         <v>-1.646922669478362</v>
       </c>
       <c r="U58">
-        <v>1.83652995004864</v>
+        <v>1.83652995031639</v>
       </c>
       <c r="V58" t="inlineStr">
         <is>
@@ -16085,6 +16208,9 @@
       <c r="C59">
         <v>65.10329204999999</v>
       </c>
+      <c r="E59">
+        <v>1189.70586264</v>
+      </c>
       <c r="G59">
         <v>19009</v>
       </c>
@@ -16121,16 +16247,16 @@
         <v>8.952</v>
       </c>
       <c r="R59">
-        <v>-1.674761726827512</v>
+        <v>-1.674761706576233</v>
       </c>
       <c r="S59">
-        <v>2.468434270800502</v>
+        <v>2.468434301342524</v>
       </c>
       <c r="T59">
         <v>-0.9328220578580235</v>
       </c>
       <c r="U59">
-        <v>1.63387809069927</v>
+        <v>1.633878091611323</v>
       </c>
       <c r="V59" t="inlineStr">
         <is>
@@ -16194,16 +16320,16 @@
         <v>6.065</v>
       </c>
       <c r="R60">
-        <v>-1.666570512078674</v>
+        <v>-1.666570492436643</v>
       </c>
       <c r="S60">
-        <v>0.6510301410178598</v>
+        <v>0.6510301531044798</v>
       </c>
       <c r="T60">
         <v>-0.9914788346738107</v>
       </c>
       <c r="U60">
-        <v>1.679720570480437</v>
+        <v>1.67972057124674</v>
       </c>
       <c r="V60" t="inlineStr">
         <is>
@@ -16267,16 +16393,16 @@
         <v>3.479</v>
       </c>
       <c r="R61">
-        <v>-1.638420075640451</v>
+        <v>-1.638420058092197</v>
       </c>
       <c r="S61">
-        <v>-0.7490148836049225</v>
+        <v>-0.7490148857354996</v>
       </c>
       <c r="T61">
         <v>0.08836358695496438</v>
       </c>
       <c r="U61">
-        <v>0.767172543982375</v>
+        <v>0.7671725476499959</v>
       </c>
       <c r="V61" t="inlineStr">
         <is>
@@ -16349,16 +16475,16 @@
         <v>4.764</v>
       </c>
       <c r="R62">
-        <v>-1.553808122130188</v>
+        <v>-1.553808110875215</v>
       </c>
       <c r="S62">
-        <v>-1.024980268931819</v>
+        <v>-1.024980273864774</v>
       </c>
       <c r="T62">
         <v>-0.203899119519819</v>
       </c>
       <c r="U62">
-        <v>0.4729570676102677</v>
+        <v>0.472957072213305</v>
       </c>
       <c r="V62" t="inlineStr">
         <is>
@@ -16422,16 +16548,16 @@
         <v>4.361</v>
       </c>
       <c r="R63">
-        <v>-1.612200648002335</v>
+        <v>-1.612200632404234</v>
       </c>
       <c r="S63">
-        <v>-0.8173591849484841</v>
+        <v>-0.8173591877730848</v>
       </c>
       <c r="T63">
         <v>-1.531804152551405</v>
       </c>
       <c r="U63">
-        <v>1.045663812688375</v>
+        <v>1.045663815470572</v>
       </c>
       <c r="V63" t="inlineStr">
         <is>
@@ -16495,16 +16621,16 @@
         <v>3.823</v>
       </c>
       <c r="R64">
-        <v>-1.59483960029272</v>
+        <v>-1.594839585985901</v>
       </c>
       <c r="S64">
-        <v>-0.9827098069246233</v>
+        <v>-0.9827098114283287</v>
       </c>
       <c r="T64">
         <v>-1.125073704945155</v>
       </c>
       <c r="U64">
-        <v>0.84735665354414</v>
+        <v>0.8473566569568267</v>
       </c>
       <c r="V64" t="inlineStr">
         <is>
@@ -16532,6 +16658,9 @@
       <c r="C65">
         <v>60.58287962</v>
       </c>
+      <c r="E65">
+        <v>1417.14408657</v>
+      </c>
       <c r="G65">
         <v>121207</v>
       </c>
@@ -16568,16 +16697,16 @@
         <v>4.131</v>
       </c>
       <c r="R65">
-        <v>-1.507236058446129</v>
+        <v>-1.5072360506551</v>
       </c>
       <c r="S65">
-        <v>-1.168649671133767</v>
+        <v>-1.168649677525657</v>
       </c>
       <c r="T65">
         <v>-1.290428149914473</v>
       </c>
       <c r="U65">
-        <v>0.3969182989471045</v>
+        <v>0.3969183037918963</v>
       </c>
       <c r="V65" t="inlineStr">
         <is>
@@ -16641,16 +16770,16 @@
         <v>5.048</v>
       </c>
       <c r="R66">
-        <v>-1.22219424330785</v>
+        <v>-1.222194256717705</v>
       </c>
       <c r="S66">
-        <v>-1.309984598235869</v>
+        <v>-1.309984606062989</v>
       </c>
       <c r="T66">
         <v>-0.8306410282985272</v>
       </c>
       <c r="U66">
-        <v>-0.12392389291387</v>
+        <v>-0.1239238864131341</v>
       </c>
       <c r="V66" t="inlineStr">
         <is>
@@ -16714,16 +16843,16 @@
         <v>7.15</v>
       </c>
       <c r="R67">
-        <v>-1.019974346357494</v>
+        <v>-1.019974374808091</v>
       </c>
       <c r="S67">
-        <v>-1.310149563079759</v>
+        <v>-1.310149570908554</v>
       </c>
       <c r="T67">
         <v>-0.326140511737147</v>
       </c>
       <c r="U67">
-        <v>-0.2508099520732978</v>
+        <v>-0.2508099451691457</v>
       </c>
       <c r="V67" t="inlineStr">
         <is>
@@ -16751,6 +16880,9 @@
       <c r="C68">
         <v>78.07311692</v>
       </c>
+      <c r="E68">
+        <v>4572.52438757</v>
+      </c>
       <c r="G68">
         <v>543733</v>
       </c>
@@ -16787,16 +16919,16 @@
         <v>10.191</v>
       </c>
       <c r="R68">
-        <v>-0.814620248366557</v>
+        <v>-0.8146202920910127</v>
       </c>
       <c r="S68">
-        <v>-1.296361335558131</v>
+        <v>-1.296361343246909</v>
       </c>
       <c r="T68">
         <v>0.09321007045758994</v>
       </c>
       <c r="U68">
-        <v>-0.2922371040346133</v>
+        <v>-0.2922370969987494</v>
       </c>
       <c r="V68" t="inlineStr">
         <is>
@@ -16860,16 +16992,16 @@
         <v>16.622</v>
       </c>
       <c r="R69">
-        <v>-0.5146319661320385</v>
+        <v>-0.5146320321690685</v>
       </c>
       <c r="S69">
-        <v>-1.261981543304708</v>
+        <v>-1.261981550644366</v>
       </c>
       <c r="T69">
         <v>0.1776985730230466</v>
       </c>
       <c r="U69">
-        <v>-0.3498865877275207</v>
+        <v>-0.3498865805083684</v>
       </c>
       <c r="V69" t="inlineStr">
         <is>
@@ -16933,16 +17065,16 @@
         <v>14.735</v>
       </c>
       <c r="R70">
-        <v>-0.5113453170282921</v>
+        <v>-0.511345383309777</v>
       </c>
       <c r="S70">
-        <v>-1.284063798435715</v>
+        <v>-1.284063805999615</v>
       </c>
       <c r="T70">
         <v>0.0197601186544395</v>
       </c>
       <c r="U70">
-        <v>-0.3756540018407054</v>
+        <v>-0.3756539945396293</v>
       </c>
       <c r="V70" t="inlineStr">
         <is>
@@ -16970,6 +17102,9 @@
       <c r="C71">
         <v>82.84273883</v>
       </c>
+      <c r="E71">
+        <v>9083.61939613</v>
+      </c>
       <c r="G71">
         <v>782215</v>
       </c>
@@ -17006,16 +17141,16 @@
         <v>14.127</v>
       </c>
       <c r="R71">
-        <v>-0.4236942376136175</v>
+        <v>-0.4236943104144278</v>
       </c>
       <c r="S71">
-        <v>-1.302042786686155</v>
+        <v>-1.302042794432627</v>
       </c>
       <c r="T71">
         <v>0.4705309185515145</v>
       </c>
       <c r="U71">
-        <v>-0.4256117572639205</v>
+        <v>-0.4256117498040108</v>
       </c>
       <c r="V71" t="inlineStr">
         <is>
@@ -17079,16 +17214,16 @@
         <v>14.971</v>
       </c>
       <c r="R72">
-        <v>-0.3669474951330728</v>
+        <v>-0.3669475721546009</v>
       </c>
       <c r="S72">
-        <v>-1.299812745140723</v>
+        <v>-1.29981275286455</v>
       </c>
       <c r="T72">
         <v>0.5962791524044461</v>
       </c>
       <c r="U72">
-        <v>-0.4252715902155837</v>
+        <v>-0.4252715827567555</v>
       </c>
       <c r="V72" t="inlineStr">
         <is>
@@ -17152,16 +17287,16 @@
         <v>16.024</v>
       </c>
       <c r="R73">
-        <v>-0.3677556337905027</v>
+        <v>-0.367755710751923</v>
       </c>
       <c r="S73">
-        <v>-1.288981299348691</v>
+        <v>-1.288981306962526</v>
       </c>
       <c r="T73">
         <v>0.7062456052859398</v>
       </c>
       <c r="U73">
-        <v>-0.4496168213667325</v>
+        <v>-0.4496168138305021</v>
       </c>
       <c r="V73" t="inlineStr">
         <is>
@@ -17234,16 +17369,16 @@
         <v>19.685</v>
       </c>
       <c r="R74">
-        <v>-0.1790790260646614</v>
+        <v>-0.1790791170594992</v>
       </c>
       <c r="S74">
-        <v>-1.276452485797809</v>
+        <v>-1.276452493284417</v>
       </c>
       <c r="T74">
         <v>0.1010946381426008</v>
       </c>
       <c r="U74">
-        <v>-0.4478043935152357</v>
+        <v>-0.4478043859847676</v>
       </c>
       <c r="V74" t="inlineStr">
         <is>
@@ -17307,16 +17442,16 @@
         <v>28.375</v>
       </c>
       <c r="R75">
-        <v>-0.1784675945855106</v>
+        <v>-0.1784676856258255</v>
       </c>
       <c r="S75">
-        <v>-1.198878737857223</v>
+        <v>-1.198878744556084</v>
       </c>
       <c r="T75">
         <v>-0.4447798235757627</v>
       </c>
       <c r="U75">
-        <v>-0.4318697922519632</v>
+        <v>-0.4318697847721569</v>
       </c>
       <c r="V75" t="inlineStr">
         <is>
@@ -17380,16 +17515,16 @@
         <v>35.312</v>
       </c>
       <c r="R76">
-        <v>-0.1357985291638057</v>
+        <v>-0.1357986233777669</v>
       </c>
       <c r="S76">
-        <v>-1.145471561494286</v>
+        <v>-1.145471567650807</v>
       </c>
       <c r="T76">
         <v>0.6481430103823895</v>
       </c>
       <c r="U76">
-        <v>-0.4861857041085468</v>
+        <v>-0.4861856964560508</v>
       </c>
       <c r="V76" t="inlineStr">
         <is>
@@ -17417,6 +17552,9 @@
       <c r="C77">
         <v>80.04863102</v>
       </c>
+      <c r="E77">
+        <v>6017.94372289</v>
+      </c>
       <c r="G77">
         <v>1021040</v>
       </c>
@@ -17453,16 +17591,16 @@
         <v>60.888</v>
       </c>
       <c r="R77">
-        <v>-0.03220597217609698</v>
+        <v>-0.03220607409508117</v>
       </c>
       <c r="S77">
-        <v>-0.955919839010503</v>
+        <v>-0.9559198432421613</v>
       </c>
       <c r="T77">
         <v>0.2494913585132937</v>
       </c>
       <c r="U77">
-        <v>-0.4849529205404556</v>
+        <v>-0.4849529128918791</v>
       </c>
       <c r="V77" t="inlineStr">
         <is>
@@ -17526,16 +17664,16 @@
         <v>90.72499999999999</v>
       </c>
       <c r="R78">
-        <v>0.1441256208862461</v>
+        <v>0.1441255058520438</v>
       </c>
       <c r="S78">
-        <v>-0.7831360546202116</v>
+        <v>-0.7831360570972827</v>
       </c>
       <c r="T78">
         <v>0.1644941167182394</v>
       </c>
       <c r="U78">
-        <v>-0.4895324426822463</v>
+        <v>-0.4895324350191098</v>
       </c>
       <c r="V78" t="inlineStr">
         <is>
@@ -17599,16 +17737,16 @@
         <v>95.613</v>
       </c>
       <c r="R79">
-        <v>0.1177373529201068</v>
+        <v>0.1177372398486151</v>
       </c>
       <c r="S79">
-        <v>-0.7368716470628386</v>
+        <v>-0.7368716490701033</v>
       </c>
       <c r="T79">
         <v>0.3028937894507765</v>
       </c>
       <c r="U79">
-        <v>-0.4795054100078674</v>
+        <v>-0.4795054023766104</v>
       </c>
       <c r="V79" t="inlineStr">
         <is>
@@ -17636,6 +17774,9 @@
       <c r="C80">
         <v>81.06717027000001</v>
       </c>
+      <c r="E80">
+        <v>12445.99017278</v>
+      </c>
       <c r="G80">
         <v>1129310</v>
       </c>
@@ -17672,16 +17813,16 @@
         <v>113.29</v>
       </c>
       <c r="R80">
-        <v>0.1452730794262074</v>
+        <v>0.1452729643066593</v>
       </c>
       <c r="S80">
-        <v>-0.6171941093765199</v>
+        <v>-0.6171941101684815</v>
       </c>
       <c r="T80">
         <v>0.3300671569473778</v>
       </c>
       <c r="U80">
-        <v>-0.4642418006450891</v>
+        <v>-0.4642417930623606</v>
       </c>
       <c r="V80" t="inlineStr">
         <is>
@@ -17745,16 +17886,16 @@
         <v>231.331</v>
       </c>
       <c r="R81">
-        <v>0.6211929834605682</v>
+        <v>0.6211928329429768</v>
       </c>
       <c r="S81">
-        <v>-0.09573887474223457</v>
+        <v>-0.09573887023891518</v>
       </c>
       <c r="T81">
         <v>1.060104594026476</v>
       </c>
       <c r="U81">
-        <v>-0.4829098102677074</v>
+        <v>-0.4829098026256265</v>
       </c>
       <c r="V81" t="inlineStr">
         <is>
@@ -17818,16 +17959,16 @@
         <v>215.442</v>
       </c>
       <c r="R82">
-        <v>0.4458793500458194</v>
+        <v>0.4458792125677322</v>
       </c>
       <c r="S82">
-        <v>-0.08598191408182367</v>
+        <v>-0.08598190947942418</v>
       </c>
       <c r="T82">
         <v>0.7419548779381776</v>
       </c>
       <c r="U82">
-        <v>-0.4643127870653763</v>
+        <v>-0.4643127794824222</v>
       </c>
       <c r="V82" t="inlineStr">
         <is>
@@ -17855,6 +17996,9 @@
       <c r="C83">
         <v>82.67366269</v>
       </c>
+      <c r="E83">
+        <v>20307.57071465</v>
+      </c>
       <c r="G83">
         <v>1130762</v>
       </c>
@@ -17891,16 +18035,16 @@
         <v>135.677</v>
       </c>
       <c r="R83">
-        <v>0.1476532362833844</v>
+        <v>0.1476531209868045</v>
       </c>
       <c r="S83">
-        <v>-0.4534340140779896</v>
+        <v>-0.4534340132069978</v>
       </c>
       <c r="T83">
         <v>0.4571554448261249</v>
       </c>
       <c r="U83">
-        <v>-0.4998304999598945</v>
+        <v>-0.4998304922640168</v>
       </c>
       <c r="V83" t="inlineStr">
         <is>
@@ -17964,16 +18108,16 @@
         <v>122.765</v>
       </c>
       <c r="R84">
-        <v>0.1397882276051923</v>
+        <v>0.1397881128935972</v>
       </c>
       <c r="S84">
-        <v>-0.5446516539260627</v>
+        <v>-0.5446516539813692</v>
       </c>
       <c r="T84">
         <v>0.06125457635334063</v>
       </c>
       <c r="U84">
-        <v>-0.5100608388020835</v>
+        <v>-0.5100608310736799</v>
       </c>
       <c r="V84" t="inlineStr">
         <is>
@@ -18037,16 +18181,16 @@
         <v>104.347</v>
       </c>
       <c r="R85">
-        <v>0.09797975608845842</v>
+        <v>0.09797964448650026</v>
       </c>
       <c r="S85">
-        <v>-0.6629564881645664</v>
+        <v>-0.6629564894212364</v>
       </c>
       <c r="T85">
         <v>0.1107764119908667</v>
       </c>
       <c r="U85">
-        <v>-0.5240596880889533</v>
+        <v>-0.5240596803160423</v>
       </c>
       <c r="V85" t="inlineStr">
         <is>
@@ -18119,16 +18263,16 @@
         <v>130.156</v>
       </c>
       <c r="R86">
-        <v>0.3128921837172727</v>
+        <v>0.3128920561305252</v>
       </c>
       <c r="S86">
-        <v>-0.5725225965899172</v>
+        <v>-0.5725225969282479</v>
       </c>
       <c r="T86">
         <v>-0.2330398957757668</v>
       </c>
       <c r="U86">
-        <v>-0.510492899830537</v>
+        <v>-0.5104928921007597</v>
       </c>
       <c r="V86" t="inlineStr">
         <is>
@@ -18192,16 +18336,16 @@
         <v>211.15</v>
       </c>
       <c r="R87">
-        <v>0.6217077005770651</v>
+        <v>0.62170755002119</v>
       </c>
       <c r="S87">
-        <v>-0.2143665091085249</v>
+        <v>-0.2143665058098471</v>
       </c>
       <c r="T87">
         <v>0.0884169516302577</v>
       </c>
       <c r="U87">
-        <v>-0.5160602035150291</v>
+        <v>-0.5160601957675514</v>
       </c>
       <c r="V87" t="inlineStr">
         <is>
@@ -18265,16 +18409,16 @@
         <v>326.86</v>
       </c>
       <c r="R88">
-        <v>0.6181850028593838</v>
+        <v>0.6181848525655205</v>
       </c>
       <c r="S88">
-        <v>0.4669829242901131</v>
+        <v>0.4669829345077677</v>
       </c>
       <c r="T88">
         <v>0.4981242283946176</v>
       </c>
       <c r="U88">
-        <v>-0.5151898991973664</v>
+        <v>-0.5151898914526556</v>
       </c>
       <c r="V88" t="inlineStr">
         <is>
@@ -18302,6 +18446,9 @@
       <c r="C89">
         <v>83.41271879</v>
       </c>
+      <c r="E89">
+        <v>8077.16805887</v>
+      </c>
       <c r="G89">
         <v>1464865</v>
       </c>
@@ -18338,16 +18485,16 @@
         <v>247.622</v>
       </c>
       <c r="R89">
-        <v>0.695323722821527</v>
+        <v>0.6953235667902281</v>
       </c>
       <c r="S89">
-        <v>-0.04503067546912503</v>
+        <v>-0.04503067045087332</v>
       </c>
       <c r="T89">
         <v>0.5156215622045961</v>
       </c>
       <c r="U89">
-        <v>-0.532001070624446</v>
+        <v>-0.5320010628262866</v>
       </c>
       <c r="V89" t="inlineStr">
         <is>
@@ -18411,16 +18558,16 @@
         <v>220.332</v>
       </c>
       <c r="R90">
-        <v>0.4960823003956132</v>
+        <v>0.4960821591835232</v>
       </c>
       <c r="S90">
-        <v>-0.08682732836849542</v>
+        <v>-0.08682732377468096</v>
       </c>
       <c r="T90">
         <v>0.08495987757582081</v>
       </c>
       <c r="U90">
-        <v>-0.5223641003787404</v>
+        <v>-0.5223640926112203</v>
       </c>
       <c r="V90" t="inlineStr">
         <is>
@@ -18484,16 +18631,16 @@
         <v>222.01</v>
       </c>
       <c r="R91">
-        <v>0.3876327153308967</v>
+        <v>0.3876325821850865</v>
       </c>
       <c r="S91">
-        <v>-0.00514940210231517</v>
+        <v>-0.00514939667907655</v>
       </c>
       <c r="T91">
         <v>0.1478216273651635</v>
       </c>
       <c r="U91">
-        <v>-0.4949456883021701</v>
+        <v>-0.4949456806218229</v>
       </c>
       <c r="V91" t="inlineStr">
         <is>
@@ -18521,6 +18668,9 @@
       <c r="C92">
         <v>76.91959518</v>
       </c>
+      <c r="E92">
+        <v>14923.35371873</v>
+      </c>
       <c r="G92">
         <v>1250293</v>
       </c>
@@ -18557,16 +18707,16 @@
         <v>216.17</v>
       </c>
       <c r="R92">
-        <v>0.3435916173406952</v>
+        <v>0.3435914874705805</v>
       </c>
       <c r="S92">
-        <v>-0.012938274164175</v>
+        <v>-0.01293826882003093</v>
       </c>
       <c r="T92">
         <v>0.001955918777550256</v>
       </c>
       <c r="U92">
-        <v>-0.485350518905447</v>
+        <v>-0.4853505112556063</v>
       </c>
       <c r="V92" t="inlineStr">
         <is>
@@ -18630,16 +18780,16 @@
         <v>412.805</v>
       </c>
       <c r="R93">
-        <v>0.9211075005032321</v>
+        <v>0.921107327678553</v>
       </c>
       <c r="S93">
-        <v>0.6921496802949879</v>
+        <v>0.692149692799169</v>
       </c>
       <c r="T93">
         <v>0.988160112740228</v>
       </c>
       <c r="U93">
-        <v>-0.4987349248652265</v>
+        <v>-0.498734917172832</v>
       </c>
       <c r="V93" t="inlineStr">
         <is>
@@ -18703,16 +18853,16 @@
         <v>403.138</v>
       </c>
       <c r="R94">
-        <v>0.8182050578659857</v>
+        <v>0.8182048926950002</v>
       </c>
       <c r="S94">
-        <v>0.7273097086215949</v>
+        <v>0.7273097214828196</v>
       </c>
       <c r="T94">
         <v>0.8665166086714168</v>
       </c>
       <c r="U94">
-        <v>-0.4953837256859098</v>
+        <v>-0.49538371800417</v>
       </c>
       <c r="V94" t="inlineStr">
         <is>
@@ -18740,6 +18890,9 @@
       <c r="C95">
         <v>83.09800989</v>
       </c>
+      <c r="E95">
+        <v>22421.03985439</v>
+      </c>
       <c r="G95">
         <v>1270681</v>
       </c>
@@ -18776,16 +18929,16 @@
         <v>217.205</v>
       </c>
       <c r="R95">
-        <v>0.3770121669303118</v>
+        <v>0.3770120345744384</v>
       </c>
       <c r="S95">
-        <v>-0.02925300615054294</v>
+        <v>-0.02925300097207194</v>
       </c>
       <c r="T95">
         <v>0.49072520117402</v>
       </c>
       <c r="U95">
-        <v>-0.5099597708158989</v>
+        <v>-0.5099597630878165</v>
       </c>
       <c r="V95" t="inlineStr">
         <is>
@@ -18849,16 +19002,16 @@
         <v>234.528</v>
       </c>
       <c r="R96">
-        <v>0.4488299577200057</v>
+        <v>0.4488298200224577</v>
       </c>
       <c r="S96">
-        <v>0.03303269654641465</v>
+        <v>0.03303270235738538</v>
       </c>
       <c r="T96">
         <v>0.3389741940893514</v>
       </c>
       <c r="U96">
-        <v>-0.5168547764125991</v>
+        <v>-0.5168547686625952</v>
       </c>
       <c r="V96" t="inlineStr">
         <is>
@@ -18922,16 +19075,16 @@
         <v>174.751</v>
       </c>
       <c r="R97">
-        <v>0.3180278802968425</v>
+        <v>0.3180277523281114</v>
       </c>
       <c r="S97">
-        <v>-0.274048091700615</v>
+        <v>-0.2740480890079926</v>
       </c>
       <c r="T97">
         <v>0.3811443493467305</v>
       </c>
       <c r="U97">
-        <v>-0.5117495225630632</v>
+        <v>-0.5117495148292907</v>
       </c>
       <c r="V97" t="inlineStr">
         <is>
@@ -19004,16 +19157,16 @@
         <v>193.483</v>
       </c>
       <c r="R98">
-        <v>0.5736537761499704</v>
+        <v>0.5736536291682574</v>
       </c>
       <c r="S98">
-        <v>-0.2940392639237111</v>
+        <v>-0.2940392614340953</v>
       </c>
       <c r="T98">
         <v>-0.1409796603793633</v>
       </c>
       <c r="U98">
-        <v>-0.5156711695943693</v>
+        <v>-0.5156711618481283</v>
       </c>
       <c r="V98" t="inlineStr">
         <is>
@@ -19036,7 +19189,7 @@
         <v>45658</v>
       </c>
       <c r="B99">
-        <v>3.52215423</v>
+        <v>3.52215261</v>
       </c>
       <c r="C99">
         <v>81.80868991</v>
@@ -19068,7 +19221,7 @@
         <v>23.04757590320142</v>
       </c>
       <c r="O99">
-        <v>3.52215423</v>
+        <v>3.52215261</v>
       </c>
       <c r="P99">
         <v>1.633495</v>
@@ -19077,16 +19230,16 @@
         <v>376.481</v>
       </c>
       <c r="R99">
-        <v>0.9717464850982112</v>
+        <v>0.9717463085070979</v>
       </c>
       <c r="S99">
-        <v>0.466455274236631</v>
+        <v>0.4664552844489274</v>
       </c>
       <c r="T99">
         <v>0.3887281629395905</v>
       </c>
       <c r="U99">
-        <v>-0.5132650021088102</v>
+        <v>-0.5132651595023281</v>
       </c>
       <c r="V99" t="inlineStr">
         <is>
@@ -19109,7 +19262,7 @@
         <v>45689</v>
       </c>
       <c r="B100">
-        <v>3.46523629</v>
+        <v>3.46523707</v>
       </c>
       <c r="C100">
         <v>83.82109185</v>
@@ -19141,7 +19294,7 @@
         <v>19.45346432302272</v>
       </c>
       <c r="O100">
-        <v>3.46523629</v>
+        <v>3.46523707</v>
       </c>
       <c r="P100">
         <v>1.377513</v>
@@ -19150,16 +19303,16 @@
         <v>267.974</v>
       </c>
       <c r="R100">
-        <v>0.5521340108462385</v>
+        <v>0.5521338654651258</v>
       </c>
       <c r="S100">
-        <v>0.1672219720920418</v>
+        <v>0.1672219792656796</v>
       </c>
       <c r="T100">
         <v>0.5479276175367497</v>
       </c>
       <c r="U100">
-        <v>-0.5190668412971023</v>
+        <v>-0.5190667540320131</v>
       </c>
       <c r="V100" t="inlineStr">
         <is>
@@ -19187,6 +19340,9 @@
       <c r="C101">
         <v>76.14225854999999</v>
       </c>
+      <c r="E101">
+        <v>8008.93668644</v>
+      </c>
       <c r="G101">
         <v>1296605</v>
       </c>
@@ -19223,16 +19379,16 @@
         <v>187.036</v>
       </c>
       <c r="R101">
-        <v>0.4195074743445367</v>
+        <v>0.4195073388279409</v>
       </c>
       <c r="S101">
-        <v>-0.2514259002062494</v>
+        <v>-0.2514258972839029</v>
       </c>
       <c r="T101">
         <v>-0.05953853969747724</v>
       </c>
       <c r="U101">
-        <v>-0.5191623365842677</v>
+        <v>-0.5191623288269271</v>
       </c>
       <c r="V101" t="inlineStr">
         <is>
@@ -19296,16 +19452,16 @@
         <v>207.505</v>
       </c>
       <c r="R102">
-        <v>0.5949686381429948</v>
+        <v>0.5949684895759217</v>
       </c>
       <c r="S102">
-        <v>-0.2215991878858073</v>
+        <v>-0.221599184660576</v>
       </c>
       <c r="T102">
         <v>0.1299913538957186</v>
       </c>
       <c r="U102">
-        <v>-0.5225644861546189</v>
+        <v>-0.5225644783864617</v>
       </c>
       <c r="V102" t="inlineStr">
         <is>
@@ -19328,7 +19484,7 @@
         <v>45778</v>
       </c>
       <c r="B103">
-        <v>3.56004101</v>
+        <v>3.56003864</v>
       </c>
       <c r="C103">
         <v>79.57640013</v>
@@ -19360,7 +19516,7 @@
         <v>17.61157644250711</v>
       </c>
       <c r="O103">
-        <v>3.56004101</v>
+        <v>3.56003864</v>
       </c>
       <c r="P103">
         <v>1.37417</v>
@@ -19369,16 +19525,16 @@
         <v>242.013</v>
       </c>
       <c r="R103">
-        <v>0.5466540767046802</v>
+        <v>0.5466539317311551</v>
       </c>
       <c r="S103">
-        <v>0.0138727561950266</v>
+        <v>0.0138727618114317</v>
       </c>
       <c r="T103">
         <v>0.2121335630164697</v>
       </c>
       <c r="U103">
-        <v>-0.5094030737796718</v>
+        <v>-0.5094033076355184</v>
       </c>
       <c r="V103" t="inlineStr">
         <is>
@@ -19406,6 +19562,9 @@
       <c r="C104">
         <v>75.02096415</v>
       </c>
+      <c r="E104">
+        <v>15594.03060042</v>
+      </c>
       <c r="G104">
         <v>1245947</v>
       </c>
@@ -19442,16 +19601,16 @@
         <v>197.185</v>
       </c>
       <c r="R104">
-        <v>0.336467539034021</v>
+        <v>0.3364674096937821</v>
       </c>
       <c r="S104">
-        <v>-0.1347786233950126</v>
+        <v>-0.1347786192881346</v>
       </c>
       <c r="T104">
         <v>-0.1482432131400242</v>
       </c>
       <c r="U104">
-        <v>-0.4947860371519022</v>
+        <v>-0.4947860294720626</v>
       </c>
       <c r="V104" t="inlineStr">
         <is>
@@ -19515,16 +19674,16 @@
         <v>414.488</v>
       </c>
       <c r="R105">
-        <v>1.049242556434228</v>
+        <v>1.0492423740791</v>
       </c>
       <c r="S105">
-        <v>0.6007490266765024</v>
+        <v>0.6007490382525269</v>
       </c>
       <c r="T105">
         <v>1.135710779484552</v>
       </c>
       <c r="U105">
-        <v>-0.5163519634106801</v>
+        <v>-0.5163519556622748</v>
       </c>
       <c r="V105" t="inlineStr">
         <is>
@@ -19588,16 +19747,16 @@
         <v>398.206</v>
       </c>
       <c r="R106">
-        <v>0.9321181848074038</v>
+        <v>0.9321180111637704</v>
       </c>
       <c r="S106">
-        <v>0.6076722564883712</v>
+        <v>0.6076722681346998</v>
       </c>
       <c r="T106">
         <v>1.001920042018988</v>
       </c>
       <c r="U106">
-        <v>-0.5044843580535214</v>
+        <v>-0.5044843503428474</v>
       </c>
       <c r="V106" t="inlineStr">
         <is>
@@ -19625,6 +19784,9 @@
       <c r="C107">
         <v>80.96374383</v>
       </c>
+      <c r="E107">
+        <v>23881.41968916</v>
+      </c>
       <c r="G107">
         <v>1254346</v>
       </c>
@@ -19661,16 +19823,16 @@
         <v>207.028</v>
       </c>
       <c r="R107">
-        <v>0.3502354022870713</v>
+        <v>0.3502352719228042</v>
       </c>
       <c r="S107">
-        <v>-0.07826896785178129</v>
+        <v>-0.07826896317105826</v>
       </c>
       <c r="T107">
         <v>0.3218851767417103</v>
       </c>
       <c r="U107">
-        <v>-0.5271418595403218</v>
+        <v>-0.5271418517576114</v>
       </c>
       <c r="V107" t="inlineStr">
         <is>
@@ -19734,16 +19896,16 @@
         <v>226.01</v>
       </c>
       <c r="R108">
-        <v>0.5546977610698092</v>
+        <v>0.5546976154980096</v>
       </c>
       <c r="S108">
-        <v>-0.08795656528908329</v>
+        <v>-0.08795656070673601</v>
       </c>
       <c r="T108">
         <v>0.6171438749897464</v>
       </c>
       <c r="U108">
-        <v>-0.5280301326778698</v>
+        <v>-0.5280301248923354</v>
       </c>
       <c r="V108" t="inlineStr">
         <is>
@@ -19772,10 +19934,10 @@
         <v>84.95384722999999</v>
       </c>
       <c r="G109">
-        <v>1293401</v>
+        <v>1293402</v>
       </c>
       <c r="H109">
-        <v>203531</v>
+        <v>203532</v>
       </c>
       <c r="I109">
         <v>2025</v>
@@ -19792,31 +19954,31 @@
         </is>
       </c>
       <c r="M109">
-        <v>0.1573610968292123</v>
+        <v>0.157361748319548</v>
       </c>
       <c r="N109">
-        <v>15.73610968292123</v>
+        <v>15.7361748319548</v>
       </c>
       <c r="O109">
         <v>3.29827077</v>
       </c>
       <c r="P109">
-        <v>1.293401</v>
+        <v>1.293402</v>
       </c>
       <c r="Q109">
-        <v>203.531</v>
+        <v>203.532</v>
       </c>
       <c r="R109">
-        <v>0.4142553926844852</v>
+        <v>0.4142568967848932</v>
       </c>
       <c r="S109">
-        <v>-0.1422721210615093</v>
+        <v>-0.142266692947414</v>
       </c>
       <c r="T109">
         <v>0.6375389596367261</v>
       </c>
       <c r="U109">
-        <v>-0.5360862045598904</v>
+        <v>-0.5360861967487428</v>
       </c>
       <c r="V109" t="inlineStr">
         <is>
@@ -19845,7 +20007,7 @@
         <v>76.44595653</v>
       </c>
       <c r="F110">
-        <v>3.48480057</v>
+        <v>3.48480029</v>
       </c>
       <c r="G110">
         <v>1363999</v>
@@ -19883,16 +20045,16 @@
         <v>172.688</v>
       </c>
       <c r="R110">
-        <v>0.5299815041190422</v>
+        <v>0.5299813603855921</v>
       </c>
       <c r="S110">
-        <v>-0.3983434220860972</v>
+        <v>-0.3983434206556707</v>
       </c>
       <c r="T110">
         <v>-0.03551324344962109</v>
       </c>
       <c r="U110">
-        <v>-0.5184006993878163</v>
+        <v>-0.5184006916328973</v>
       </c>
       <c r="V110" t="inlineStr">
         <is>
@@ -19915,13 +20077,13 @@
         <v>46023</v>
       </c>
       <c r="B111">
-        <v>3.43209009</v>
+        <v>3.43208671</v>
       </c>
       <c r="C111">
         <v>81.17069512</v>
       </c>
       <c r="G111">
-        <v>1501420</v>
+        <v>1501426</v>
       </c>
       <c r="H111">
         <v>271953</v>
@@ -19941,31 +20103,31 @@
         </is>
       </c>
       <c r="M111">
-        <v>0.1811305297651556</v>
+        <v>0.1811298059311614</v>
       </c>
       <c r="N111">
-        <v>18.11305297651557</v>
+        <v>18.11298059311614</v>
       </c>
       <c r="O111">
-        <v>3.43209009</v>
+        <v>3.43208671</v>
       </c>
       <c r="P111">
-        <v>1.50142</v>
+        <v>1.501426</v>
       </c>
       <c r="Q111">
         <v>271.953</v>
       </c>
       <c r="R111">
-        <v>0.7552456470047932</v>
+        <v>0.7552553218747948</v>
       </c>
       <c r="S111">
-        <v>0.05562395836886446</v>
+        <v>0.05561793801764162</v>
       </c>
       <c r="T111">
         <v>0.3382569222868271</v>
       </c>
       <c r="U111">
-        <v>-0.5224455461852795</v>
+        <v>-0.5224458829523938</v>
       </c>
       <c r="V111" t="inlineStr">
         <is>

</xml_diff>